<commit_message>
data: corregir fecha de fallo incorrecta ya publicada (N0449)
El fix del extractor de fallo llega demasiado tarde para esta
licitación porque ya tenía url_pdf guardado (no se vuelve a reanalizar
el PDF una vez descargado). Se corrige el valor a mano: fallo_prog y
fallo_hora quedan en null/pendiente, como corresponde según el PDF.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/licitaciones.xlsx
+++ b/data/licitaciones.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,72 +429,72 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>No. Licitación</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Convocatoria</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Publicada</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Junta (prog.)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Hora</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Apertura (prog.)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Hora</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Fallo (prog.)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Hora</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Acta Junta</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Acta Apertura</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Acta Fallo</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Objeto</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>PDF</t>
         </is>
@@ -18512,16 +18524,8 @@
           <t>12:00</t>
         </is>
       </c>
-      <c r="H450" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="I450" t="inlineStr">
-        <is>
-          <t>10:00</t>
-        </is>
-      </c>
+      <c r="H450" t="inlineStr"/>
+      <c r="I450" t="inlineStr"/>
       <c r="J450" t="inlineStr"/>
       <c r="K450" t="inlineStr"/>
       <c r="L450" t="inlineStr"/>

</xml_diff>

<commit_message>
data: rellenar objeto y solicitante para las 30 licitaciones ya procesadas
Igual que con el fix de la fecha de fallo, estas 30 licitaciones ya
tenían url_pdf guardado, así que no se iban a reanalizar solas con el
nuevo extractor. Se corrigen a mano reanalizando los PDFs que ya están
en docs/pdfs/ (sin volver a descargar nada) y regenerando el tablero
y el Excel.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/licitaciones.xlsx
+++ b/data/licitaciones.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N452"/>
+  <dimension ref="A1:O452"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -495,6 +495,11 @@
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Solicitante</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>PDF</t>
         </is>
@@ -539,6 +544,7 @@
       </c>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -579,6 +585,7 @@
       </c>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -615,6 +622,7 @@
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -655,6 +663,7 @@
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -695,6 +704,7 @@
       </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -735,6 +745,7 @@
       </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -775,6 +786,7 @@
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -815,6 +827,7 @@
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -855,6 +868,7 @@
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -895,6 +909,7 @@
       </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -935,6 +950,7 @@
       </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -975,6 +991,7 @@
       </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1015,6 +1032,7 @@
       </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1055,6 +1073,7 @@
       </c>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1095,6 +1114,7 @@
       </c>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1135,6 +1155,7 @@
       </c>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1175,6 +1196,7 @@
       </c>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1215,6 +1237,7 @@
       </c>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1255,6 +1278,7 @@
       </c>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1295,6 +1319,7 @@
       </c>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1335,6 +1360,7 @@
       </c>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1371,6 +1397,7 @@
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1411,6 +1438,7 @@
       </c>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1451,6 +1479,7 @@
       </c>
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1491,6 +1520,7 @@
       </c>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1531,6 +1561,7 @@
       </c>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1571,6 +1602,7 @@
       </c>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1611,6 +1643,7 @@
       </c>
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1651,6 +1684,7 @@
       </c>
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1691,6 +1725,7 @@
       </c>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1731,6 +1766,7 @@
       </c>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1771,6 +1807,7 @@
       </c>
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1811,6 +1848,7 @@
       </c>
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1847,6 +1885,7 @@
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1887,6 +1926,7 @@
       </c>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1927,6 +1967,7 @@
       </c>
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1967,6 +2008,7 @@
       </c>
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2003,6 +2045,7 @@
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2043,6 +2086,7 @@
       </c>
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2083,6 +2127,7 @@
       </c>
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2123,6 +2168,7 @@
       </c>
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2163,6 +2209,7 @@
       </c>
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2199,6 +2246,7 @@
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2239,6 +2287,7 @@
       </c>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2279,6 +2328,7 @@
       </c>
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2319,6 +2369,7 @@
       </c>
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2359,6 +2410,7 @@
       </c>
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2399,6 +2451,7 @@
       </c>
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2439,6 +2492,7 @@
       </c>
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2479,6 +2533,7 @@
       </c>
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2519,6 +2574,7 @@
       </c>
       <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2559,6 +2615,7 @@
       </c>
       <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2599,6 +2656,7 @@
       </c>
       <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2635,6 +2693,7 @@
       <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr"/>
       <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2675,6 +2734,7 @@
       </c>
       <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2715,6 +2775,7 @@
       </c>
       <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2755,6 +2816,7 @@
       </c>
       <c r="M58" t="inlineStr"/>
       <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2795,6 +2857,7 @@
       </c>
       <c r="M59" t="inlineStr"/>
       <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2835,6 +2898,7 @@
       </c>
       <c r="M60" t="inlineStr"/>
       <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2875,6 +2939,7 @@
       </c>
       <c r="M61" t="inlineStr"/>
       <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2915,6 +2980,7 @@
       </c>
       <c r="M62" t="inlineStr"/>
       <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2951,6 +3017,7 @@
       <c r="L63" t="inlineStr"/>
       <c r="M63" t="inlineStr"/>
       <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2991,6 +3058,7 @@
       </c>
       <c r="M64" t="inlineStr"/>
       <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3031,6 +3099,7 @@
       </c>
       <c r="M65" t="inlineStr"/>
       <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3071,6 +3140,7 @@
       </c>
       <c r="M66" t="inlineStr"/>
       <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3111,6 +3181,7 @@
       </c>
       <c r="M67" t="inlineStr"/>
       <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3151,6 +3222,7 @@
       </c>
       <c r="M68" t="inlineStr"/>
       <c r="N68" t="inlineStr"/>
+      <c r="O68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3191,6 +3263,7 @@
       </c>
       <c r="M69" t="inlineStr"/>
       <c r="N69" t="inlineStr"/>
+      <c r="O69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3231,6 +3304,7 @@
       </c>
       <c r="M70" t="inlineStr"/>
       <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3267,6 +3341,7 @@
       <c r="L71" t="inlineStr"/>
       <c r="M71" t="inlineStr"/>
       <c r="N71" t="inlineStr"/>
+      <c r="O71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3307,6 +3382,7 @@
       </c>
       <c r="M72" t="inlineStr"/>
       <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3347,6 +3423,7 @@
       </c>
       <c r="M73" t="inlineStr"/>
       <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3387,6 +3464,7 @@
       </c>
       <c r="M74" t="inlineStr"/>
       <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3427,6 +3505,7 @@
       </c>
       <c r="M75" t="inlineStr"/>
       <c r="N75" t="inlineStr"/>
+      <c r="O75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3467,6 +3546,7 @@
       </c>
       <c r="M76" t="inlineStr"/>
       <c r="N76" t="inlineStr"/>
+      <c r="O76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3507,6 +3587,7 @@
       </c>
       <c r="M77" t="inlineStr"/>
       <c r="N77" t="inlineStr"/>
+      <c r="O77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3547,6 +3628,7 @@
       </c>
       <c r="M78" t="inlineStr"/>
       <c r="N78" t="inlineStr"/>
+      <c r="O78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3587,6 +3669,7 @@
       </c>
       <c r="M79" t="inlineStr"/>
       <c r="N79" t="inlineStr"/>
+      <c r="O79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3627,6 +3710,7 @@
       </c>
       <c r="M80" t="inlineStr"/>
       <c r="N80" t="inlineStr"/>
+      <c r="O80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3663,6 +3747,7 @@
       <c r="L81" t="inlineStr"/>
       <c r="M81" t="inlineStr"/>
       <c r="N81" t="inlineStr"/>
+      <c r="O81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3703,6 +3788,7 @@
       </c>
       <c r="M82" t="inlineStr"/>
       <c r="N82" t="inlineStr"/>
+      <c r="O82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3743,6 +3829,7 @@
       </c>
       <c r="M83" t="inlineStr"/>
       <c r="N83" t="inlineStr"/>
+      <c r="O83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3779,6 +3866,7 @@
       <c r="L84" t="inlineStr"/>
       <c r="M84" t="inlineStr"/>
       <c r="N84" t="inlineStr"/>
+      <c r="O84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3815,6 +3903,7 @@
       <c r="L85" t="inlineStr"/>
       <c r="M85" t="inlineStr"/>
       <c r="N85" t="inlineStr"/>
+      <c r="O85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3855,6 +3944,7 @@
       </c>
       <c r="M86" t="inlineStr"/>
       <c r="N86" t="inlineStr"/>
+      <c r="O86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3891,6 +3981,7 @@
       <c r="L87" t="inlineStr"/>
       <c r="M87" t="inlineStr"/>
       <c r="N87" t="inlineStr"/>
+      <c r="O87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3931,6 +4022,7 @@
       </c>
       <c r="M88" t="inlineStr"/>
       <c r="N88" t="inlineStr"/>
+      <c r="O88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3971,6 +4063,7 @@
       </c>
       <c r="M89" t="inlineStr"/>
       <c r="N89" t="inlineStr"/>
+      <c r="O89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4011,6 +4104,7 @@
       </c>
       <c r="M90" t="inlineStr"/>
       <c r="N90" t="inlineStr"/>
+      <c r="O90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4051,6 +4145,7 @@
       </c>
       <c r="M91" t="inlineStr"/>
       <c r="N91" t="inlineStr"/>
+      <c r="O91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4091,6 +4186,7 @@
       </c>
       <c r="M92" t="inlineStr"/>
       <c r="N92" t="inlineStr"/>
+      <c r="O92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4131,6 +4227,7 @@
       </c>
       <c r="M93" t="inlineStr"/>
       <c r="N93" t="inlineStr"/>
+      <c r="O93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4171,6 +4268,7 @@
       </c>
       <c r="M94" t="inlineStr"/>
       <c r="N94" t="inlineStr"/>
+      <c r="O94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4211,6 +4309,7 @@
       </c>
       <c r="M95" t="inlineStr"/>
       <c r="N95" t="inlineStr"/>
+      <c r="O95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4251,6 +4350,7 @@
       </c>
       <c r="M96" t="inlineStr"/>
       <c r="N96" t="inlineStr"/>
+      <c r="O96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4291,6 +4391,7 @@
       </c>
       <c r="M97" t="inlineStr"/>
       <c r="N97" t="inlineStr"/>
+      <c r="O97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4331,6 +4432,7 @@
       </c>
       <c r="M98" t="inlineStr"/>
       <c r="N98" t="inlineStr"/>
+      <c r="O98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4371,6 +4473,7 @@
       </c>
       <c r="M99" t="inlineStr"/>
       <c r="N99" t="inlineStr"/>
+      <c r="O99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4411,6 +4514,7 @@
       </c>
       <c r="M100" t="inlineStr"/>
       <c r="N100" t="inlineStr"/>
+      <c r="O100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -4451,6 +4555,7 @@
       </c>
       <c r="M101" t="inlineStr"/>
       <c r="N101" t="inlineStr"/>
+      <c r="O101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -4491,6 +4596,7 @@
       </c>
       <c r="M102" t="inlineStr"/>
       <c r="N102" t="inlineStr"/>
+      <c r="O102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -4531,6 +4637,7 @@
       </c>
       <c r="M103" t="inlineStr"/>
       <c r="N103" t="inlineStr"/>
+      <c r="O103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -4571,6 +4678,7 @@
       </c>
       <c r="M104" t="inlineStr"/>
       <c r="N104" t="inlineStr"/>
+      <c r="O104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -4611,6 +4719,7 @@
       </c>
       <c r="M105" t="inlineStr"/>
       <c r="N105" t="inlineStr"/>
+      <c r="O105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -4651,6 +4760,7 @@
       </c>
       <c r="M106" t="inlineStr"/>
       <c r="N106" t="inlineStr"/>
+      <c r="O106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -4691,6 +4801,7 @@
       </c>
       <c r="M107" t="inlineStr"/>
       <c r="N107" t="inlineStr"/>
+      <c r="O107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -4731,6 +4842,7 @@
       </c>
       <c r="M108" t="inlineStr"/>
       <c r="N108" t="inlineStr"/>
+      <c r="O108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -4771,6 +4883,7 @@
       </c>
       <c r="M109" t="inlineStr"/>
       <c r="N109" t="inlineStr"/>
+      <c r="O109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -4807,6 +4920,7 @@
       <c r="L110" t="inlineStr"/>
       <c r="M110" t="inlineStr"/>
       <c r="N110" t="inlineStr"/>
+      <c r="O110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -4847,6 +4961,7 @@
       </c>
       <c r="M111" t="inlineStr"/>
       <c r="N111" t="inlineStr"/>
+      <c r="O111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -4887,6 +5002,7 @@
       </c>
       <c r="M112" t="inlineStr"/>
       <c r="N112" t="inlineStr"/>
+      <c r="O112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -4927,6 +5043,7 @@
       </c>
       <c r="M113" t="inlineStr"/>
       <c r="N113" t="inlineStr"/>
+      <c r="O113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -4967,6 +5084,7 @@
       </c>
       <c r="M114" t="inlineStr"/>
       <c r="N114" t="inlineStr"/>
+      <c r="O114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -5007,6 +5125,7 @@
       </c>
       <c r="M115" t="inlineStr"/>
       <c r="N115" t="inlineStr"/>
+      <c r="O115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -5047,6 +5166,7 @@
       </c>
       <c r="M116" t="inlineStr"/>
       <c r="N116" t="inlineStr"/>
+      <c r="O116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -5083,6 +5203,7 @@
       <c r="L117" t="inlineStr"/>
       <c r="M117" t="inlineStr"/>
       <c r="N117" t="inlineStr"/>
+      <c r="O117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -5123,6 +5244,7 @@
       </c>
       <c r="M118" t="inlineStr"/>
       <c r="N118" t="inlineStr"/>
+      <c r="O118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -5163,6 +5285,7 @@
       </c>
       <c r="M119" t="inlineStr"/>
       <c r="N119" t="inlineStr"/>
+      <c r="O119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -5203,6 +5326,7 @@
       </c>
       <c r="M120" t="inlineStr"/>
       <c r="N120" t="inlineStr"/>
+      <c r="O120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -5243,6 +5367,7 @@
       </c>
       <c r="M121" t="inlineStr"/>
       <c r="N121" t="inlineStr"/>
+      <c r="O121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -5283,6 +5408,7 @@
       </c>
       <c r="M122" t="inlineStr"/>
       <c r="N122" t="inlineStr"/>
+      <c r="O122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -5323,6 +5449,7 @@
       </c>
       <c r="M123" t="inlineStr"/>
       <c r="N123" t="inlineStr"/>
+      <c r="O123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -5363,6 +5490,7 @@
       </c>
       <c r="M124" t="inlineStr"/>
       <c r="N124" t="inlineStr"/>
+      <c r="O124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -5403,6 +5531,7 @@
       </c>
       <c r="M125" t="inlineStr"/>
       <c r="N125" t="inlineStr"/>
+      <c r="O125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -5443,6 +5572,7 @@
       </c>
       <c r="M126" t="inlineStr"/>
       <c r="N126" t="inlineStr"/>
+      <c r="O126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -5483,6 +5613,7 @@
       </c>
       <c r="M127" t="inlineStr"/>
       <c r="N127" t="inlineStr"/>
+      <c r="O127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -5523,6 +5654,7 @@
       </c>
       <c r="M128" t="inlineStr"/>
       <c r="N128" t="inlineStr"/>
+      <c r="O128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -5563,6 +5695,7 @@
       </c>
       <c r="M129" t="inlineStr"/>
       <c r="N129" t="inlineStr"/>
+      <c r="O129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -5599,6 +5732,7 @@
       <c r="L130" t="inlineStr"/>
       <c r="M130" t="inlineStr"/>
       <c r="N130" t="inlineStr"/>
+      <c r="O130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -5635,6 +5769,7 @@
       <c r="L131" t="inlineStr"/>
       <c r="M131" t="inlineStr"/>
       <c r="N131" t="inlineStr"/>
+      <c r="O131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -5675,6 +5810,7 @@
       </c>
       <c r="M132" t="inlineStr"/>
       <c r="N132" t="inlineStr"/>
+      <c r="O132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -5715,6 +5851,7 @@
       </c>
       <c r="M133" t="inlineStr"/>
       <c r="N133" t="inlineStr"/>
+      <c r="O133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -5755,6 +5892,7 @@
       </c>
       <c r="M134" t="inlineStr"/>
       <c r="N134" t="inlineStr"/>
+      <c r="O134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -5795,6 +5933,7 @@
       </c>
       <c r="M135" t="inlineStr"/>
       <c r="N135" t="inlineStr"/>
+      <c r="O135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -5831,6 +5970,7 @@
       <c r="L136" t="inlineStr"/>
       <c r="M136" t="inlineStr"/>
       <c r="N136" t="inlineStr"/>
+      <c r="O136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -5871,6 +6011,7 @@
       </c>
       <c r="M137" t="inlineStr"/>
       <c r="N137" t="inlineStr"/>
+      <c r="O137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -5911,6 +6052,7 @@
       </c>
       <c r="M138" t="inlineStr"/>
       <c r="N138" t="inlineStr"/>
+      <c r="O138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -5947,6 +6089,7 @@
       <c r="L139" t="inlineStr"/>
       <c r="M139" t="inlineStr"/>
       <c r="N139" t="inlineStr"/>
+      <c r="O139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -5987,6 +6130,7 @@
       </c>
       <c r="M140" t="inlineStr"/>
       <c r="N140" t="inlineStr"/>
+      <c r="O140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -6027,6 +6171,7 @@
       </c>
       <c r="M141" t="inlineStr"/>
       <c r="N141" t="inlineStr"/>
+      <c r="O141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -6067,6 +6212,7 @@
       </c>
       <c r="M142" t="inlineStr"/>
       <c r="N142" t="inlineStr"/>
+      <c r="O142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -6107,6 +6253,7 @@
       </c>
       <c r="M143" t="inlineStr"/>
       <c r="N143" t="inlineStr"/>
+      <c r="O143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -6143,6 +6290,7 @@
       <c r="L144" t="inlineStr"/>
       <c r="M144" t="inlineStr"/>
       <c r="N144" t="inlineStr"/>
+      <c r="O144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -6183,6 +6331,7 @@
       </c>
       <c r="M145" t="inlineStr"/>
       <c r="N145" t="inlineStr"/>
+      <c r="O145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -6223,6 +6372,7 @@
       </c>
       <c r="M146" t="inlineStr"/>
       <c r="N146" t="inlineStr"/>
+      <c r="O146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -6259,6 +6409,7 @@
       <c r="L147" t="inlineStr"/>
       <c r="M147" t="inlineStr"/>
       <c r="N147" t="inlineStr"/>
+      <c r="O147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -6299,6 +6450,7 @@
       </c>
       <c r="M148" t="inlineStr"/>
       <c r="N148" t="inlineStr"/>
+      <c r="O148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -6339,6 +6491,7 @@
       </c>
       <c r="M149" t="inlineStr"/>
       <c r="N149" t="inlineStr"/>
+      <c r="O149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -6375,6 +6528,7 @@
       <c r="L150" t="inlineStr"/>
       <c r="M150" t="inlineStr"/>
       <c r="N150" t="inlineStr"/>
+      <c r="O150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -6415,6 +6569,7 @@
       </c>
       <c r="M151" t="inlineStr"/>
       <c r="N151" t="inlineStr"/>
+      <c r="O151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -6455,6 +6610,7 @@
       </c>
       <c r="M152" t="inlineStr"/>
       <c r="N152" t="inlineStr"/>
+      <c r="O152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -6495,6 +6651,7 @@
       </c>
       <c r="M153" t="inlineStr"/>
       <c r="N153" t="inlineStr"/>
+      <c r="O153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -6535,6 +6692,7 @@
       </c>
       <c r="M154" t="inlineStr"/>
       <c r="N154" t="inlineStr"/>
+      <c r="O154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -6575,6 +6733,7 @@
       </c>
       <c r="M155" t="inlineStr"/>
       <c r="N155" t="inlineStr"/>
+      <c r="O155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -6615,6 +6774,7 @@
       </c>
       <c r="M156" t="inlineStr"/>
       <c r="N156" t="inlineStr"/>
+      <c r="O156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -6655,6 +6815,7 @@
       </c>
       <c r="M157" t="inlineStr"/>
       <c r="N157" t="inlineStr"/>
+      <c r="O157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -6695,6 +6856,7 @@
       </c>
       <c r="M158" t="inlineStr"/>
       <c r="N158" t="inlineStr"/>
+      <c r="O158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -6735,6 +6897,7 @@
       </c>
       <c r="M159" t="inlineStr"/>
       <c r="N159" t="inlineStr"/>
+      <c r="O159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -6775,6 +6938,7 @@
       </c>
       <c r="M160" t="inlineStr"/>
       <c r="N160" t="inlineStr"/>
+      <c r="O160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -6811,6 +6975,7 @@
       <c r="L161" t="inlineStr"/>
       <c r="M161" t="inlineStr"/>
       <c r="N161" t="inlineStr"/>
+      <c r="O161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -6851,6 +7016,7 @@
       </c>
       <c r="M162" t="inlineStr"/>
       <c r="N162" t="inlineStr"/>
+      <c r="O162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -6891,6 +7057,7 @@
       </c>
       <c r="M163" t="inlineStr"/>
       <c r="N163" t="inlineStr"/>
+      <c r="O163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -6927,6 +7094,7 @@
       <c r="L164" t="inlineStr"/>
       <c r="M164" t="inlineStr"/>
       <c r="N164" t="inlineStr"/>
+      <c r="O164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -6967,6 +7135,7 @@
       </c>
       <c r="M165" t="inlineStr"/>
       <c r="N165" t="inlineStr"/>
+      <c r="O165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -7003,6 +7172,7 @@
       <c r="L166" t="inlineStr"/>
       <c r="M166" t="inlineStr"/>
       <c r="N166" t="inlineStr"/>
+      <c r="O166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -7043,6 +7213,7 @@
       </c>
       <c r="M167" t="inlineStr"/>
       <c r="N167" t="inlineStr"/>
+      <c r="O167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -7083,6 +7254,7 @@
       </c>
       <c r="M168" t="inlineStr"/>
       <c r="N168" t="inlineStr"/>
+      <c r="O168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -7123,6 +7295,7 @@
       </c>
       <c r="M169" t="inlineStr"/>
       <c r="N169" t="inlineStr"/>
+      <c r="O169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -7163,6 +7336,7 @@
       </c>
       <c r="M170" t="inlineStr"/>
       <c r="N170" t="inlineStr"/>
+      <c r="O170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -7203,6 +7377,7 @@
       </c>
       <c r="M171" t="inlineStr"/>
       <c r="N171" t="inlineStr"/>
+      <c r="O171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -7243,6 +7418,7 @@
       </c>
       <c r="M172" t="inlineStr"/>
       <c r="N172" t="inlineStr"/>
+      <c r="O172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -7283,6 +7459,7 @@
       </c>
       <c r="M173" t="inlineStr"/>
       <c r="N173" t="inlineStr"/>
+      <c r="O173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -7323,6 +7500,7 @@
       </c>
       <c r="M174" t="inlineStr"/>
       <c r="N174" t="inlineStr"/>
+      <c r="O174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -7363,6 +7541,7 @@
       </c>
       <c r="M175" t="inlineStr"/>
       <c r="N175" t="inlineStr"/>
+      <c r="O175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -7403,6 +7582,7 @@
       </c>
       <c r="M176" t="inlineStr"/>
       <c r="N176" t="inlineStr"/>
+      <c r="O176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -7443,6 +7623,7 @@
       </c>
       <c r="M177" t="inlineStr"/>
       <c r="N177" t="inlineStr"/>
+      <c r="O177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -7479,6 +7660,7 @@
       <c r="L178" t="inlineStr"/>
       <c r="M178" t="inlineStr"/>
       <c r="N178" t="inlineStr"/>
+      <c r="O178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -7519,6 +7701,7 @@
       </c>
       <c r="M179" t="inlineStr"/>
       <c r="N179" t="inlineStr"/>
+      <c r="O179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -7559,6 +7742,7 @@
       </c>
       <c r="M180" t="inlineStr"/>
       <c r="N180" t="inlineStr"/>
+      <c r="O180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -7599,6 +7783,7 @@
       </c>
       <c r="M181" t="inlineStr"/>
       <c r="N181" t="inlineStr"/>
+      <c r="O181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -7639,6 +7824,7 @@
       </c>
       <c r="M182" t="inlineStr"/>
       <c r="N182" t="inlineStr"/>
+      <c r="O182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -7675,6 +7861,7 @@
       <c r="L183" t="inlineStr"/>
       <c r="M183" t="inlineStr"/>
       <c r="N183" t="inlineStr"/>
+      <c r="O183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -7715,6 +7902,7 @@
       </c>
       <c r="M184" t="inlineStr"/>
       <c r="N184" t="inlineStr"/>
+      <c r="O184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -7755,6 +7943,7 @@
       </c>
       <c r="M185" t="inlineStr"/>
       <c r="N185" t="inlineStr"/>
+      <c r="O185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -7795,6 +7984,7 @@
       </c>
       <c r="M186" t="inlineStr"/>
       <c r="N186" t="inlineStr"/>
+      <c r="O186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -7835,6 +8025,7 @@
       </c>
       <c r="M187" t="inlineStr"/>
       <c r="N187" t="inlineStr"/>
+      <c r="O187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -7875,6 +8066,7 @@
       </c>
       <c r="M188" t="inlineStr"/>
       <c r="N188" t="inlineStr"/>
+      <c r="O188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -7915,6 +8107,7 @@
       </c>
       <c r="M189" t="inlineStr"/>
       <c r="N189" t="inlineStr"/>
+      <c r="O189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -7955,6 +8148,7 @@
       </c>
       <c r="M190" t="inlineStr"/>
       <c r="N190" t="inlineStr"/>
+      <c r="O190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -7995,6 +8189,7 @@
       </c>
       <c r="M191" t="inlineStr"/>
       <c r="N191" t="inlineStr"/>
+      <c r="O191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -8035,6 +8230,7 @@
       </c>
       <c r="M192" t="inlineStr"/>
       <c r="N192" t="inlineStr"/>
+      <c r="O192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -8075,6 +8271,7 @@
       </c>
       <c r="M193" t="inlineStr"/>
       <c r="N193" t="inlineStr"/>
+      <c r="O193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -8115,6 +8312,7 @@
       </c>
       <c r="M194" t="inlineStr"/>
       <c r="N194" t="inlineStr"/>
+      <c r="O194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -8151,6 +8349,7 @@
       <c r="L195" t="inlineStr"/>
       <c r="M195" t="inlineStr"/>
       <c r="N195" t="inlineStr"/>
+      <c r="O195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -8191,6 +8390,7 @@
       </c>
       <c r="M196" t="inlineStr"/>
       <c r="N196" t="inlineStr"/>
+      <c r="O196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -8231,6 +8431,7 @@
       </c>
       <c r="M197" t="inlineStr"/>
       <c r="N197" t="inlineStr"/>
+      <c r="O197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -8271,6 +8472,7 @@
       </c>
       <c r="M198" t="inlineStr"/>
       <c r="N198" t="inlineStr"/>
+      <c r="O198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -8307,6 +8509,7 @@
       <c r="L199" t="inlineStr"/>
       <c r="M199" t="inlineStr"/>
       <c r="N199" t="inlineStr"/>
+      <c r="O199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -8347,6 +8550,7 @@
       </c>
       <c r="M200" t="inlineStr"/>
       <c r="N200" t="inlineStr"/>
+      <c r="O200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -8387,6 +8591,7 @@
       </c>
       <c r="M201" t="inlineStr"/>
       <c r="N201" t="inlineStr"/>
+      <c r="O201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -8427,6 +8632,7 @@
       </c>
       <c r="M202" t="inlineStr"/>
       <c r="N202" t="inlineStr"/>
+      <c r="O202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -8467,6 +8673,7 @@
       </c>
       <c r="M203" t="inlineStr"/>
       <c r="N203" t="inlineStr"/>
+      <c r="O203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -8507,6 +8714,7 @@
       </c>
       <c r="M204" t="inlineStr"/>
       <c r="N204" t="inlineStr"/>
+      <c r="O204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -8547,6 +8755,7 @@
       </c>
       <c r="M205" t="inlineStr"/>
       <c r="N205" t="inlineStr"/>
+      <c r="O205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -8587,6 +8796,7 @@
       </c>
       <c r="M206" t="inlineStr"/>
       <c r="N206" t="inlineStr"/>
+      <c r="O206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -8627,6 +8837,7 @@
       </c>
       <c r="M207" t="inlineStr"/>
       <c r="N207" t="inlineStr"/>
+      <c r="O207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -8667,6 +8878,7 @@
       </c>
       <c r="M208" t="inlineStr"/>
       <c r="N208" t="inlineStr"/>
+      <c r="O208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -8707,6 +8919,7 @@
       </c>
       <c r="M209" t="inlineStr"/>
       <c r="N209" t="inlineStr"/>
+      <c r="O209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -8747,6 +8960,7 @@
       </c>
       <c r="M210" t="inlineStr"/>
       <c r="N210" t="inlineStr"/>
+      <c r="O210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -8787,6 +9001,7 @@
       </c>
       <c r="M211" t="inlineStr"/>
       <c r="N211" t="inlineStr"/>
+      <c r="O211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -8827,6 +9042,7 @@
       </c>
       <c r="M212" t="inlineStr"/>
       <c r="N212" t="inlineStr"/>
+      <c r="O212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -8867,6 +9083,7 @@
       </c>
       <c r="M213" t="inlineStr"/>
       <c r="N213" t="inlineStr"/>
+      <c r="O213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -8907,6 +9124,7 @@
       </c>
       <c r="M214" t="inlineStr"/>
       <c r="N214" t="inlineStr"/>
+      <c r="O214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -8947,6 +9165,7 @@
       </c>
       <c r="M215" t="inlineStr"/>
       <c r="N215" t="inlineStr"/>
+      <c r="O215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -8987,6 +9206,7 @@
       </c>
       <c r="M216" t="inlineStr"/>
       <c r="N216" t="inlineStr"/>
+      <c r="O216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -9027,6 +9247,7 @@
       </c>
       <c r="M217" t="inlineStr"/>
       <c r="N217" t="inlineStr"/>
+      <c r="O217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -9067,6 +9288,7 @@
       </c>
       <c r="M218" t="inlineStr"/>
       <c r="N218" t="inlineStr"/>
+      <c r="O218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -9107,6 +9329,7 @@
       </c>
       <c r="M219" t="inlineStr"/>
       <c r="N219" t="inlineStr"/>
+      <c r="O219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -9147,6 +9370,7 @@
       </c>
       <c r="M220" t="inlineStr"/>
       <c r="N220" t="inlineStr"/>
+      <c r="O220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -9187,6 +9411,7 @@
       </c>
       <c r="M221" t="inlineStr"/>
       <c r="N221" t="inlineStr"/>
+      <c r="O221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -9227,6 +9452,7 @@
       </c>
       <c r="M222" t="inlineStr"/>
       <c r="N222" t="inlineStr"/>
+      <c r="O222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -9263,6 +9489,7 @@
       <c r="L223" t="inlineStr"/>
       <c r="M223" t="inlineStr"/>
       <c r="N223" t="inlineStr"/>
+      <c r="O223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -9303,6 +9530,7 @@
       </c>
       <c r="M224" t="inlineStr"/>
       <c r="N224" t="inlineStr"/>
+      <c r="O224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -9343,6 +9571,7 @@
       </c>
       <c r="M225" t="inlineStr"/>
       <c r="N225" t="inlineStr"/>
+      <c r="O225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -9383,6 +9612,7 @@
       </c>
       <c r="M226" t="inlineStr"/>
       <c r="N226" t="inlineStr"/>
+      <c r="O226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -9423,6 +9653,7 @@
       </c>
       <c r="M227" t="inlineStr"/>
       <c r="N227" t="inlineStr"/>
+      <c r="O227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -9463,6 +9694,7 @@
       </c>
       <c r="M228" t="inlineStr"/>
       <c r="N228" t="inlineStr"/>
+      <c r="O228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -9503,6 +9735,7 @@
       </c>
       <c r="M229" t="inlineStr"/>
       <c r="N229" t="inlineStr"/>
+      <c r="O229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -9539,6 +9772,7 @@
       <c r="L230" t="inlineStr"/>
       <c r="M230" t="inlineStr"/>
       <c r="N230" t="inlineStr"/>
+      <c r="O230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -9579,6 +9813,7 @@
       </c>
       <c r="M231" t="inlineStr"/>
       <c r="N231" t="inlineStr"/>
+      <c r="O231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -9619,6 +9854,7 @@
       </c>
       <c r="M232" t="inlineStr"/>
       <c r="N232" t="inlineStr"/>
+      <c r="O232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -9659,6 +9895,7 @@
       </c>
       <c r="M233" t="inlineStr"/>
       <c r="N233" t="inlineStr"/>
+      <c r="O233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -9699,6 +9936,7 @@
       </c>
       <c r="M234" t="inlineStr"/>
       <c r="N234" t="inlineStr"/>
+      <c r="O234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -9739,6 +9977,7 @@
       </c>
       <c r="M235" t="inlineStr"/>
       <c r="N235" t="inlineStr"/>
+      <c r="O235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -9779,6 +10018,7 @@
       </c>
       <c r="M236" t="inlineStr"/>
       <c r="N236" t="inlineStr"/>
+      <c r="O236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -9815,6 +10055,7 @@
       <c r="L237" t="inlineStr"/>
       <c r="M237" t="inlineStr"/>
       <c r="N237" t="inlineStr"/>
+      <c r="O237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -9855,6 +10096,7 @@
       </c>
       <c r="M238" t="inlineStr"/>
       <c r="N238" t="inlineStr"/>
+      <c r="O238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -9895,6 +10137,7 @@
       </c>
       <c r="M239" t="inlineStr"/>
       <c r="N239" t="inlineStr"/>
+      <c r="O239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -9935,6 +10178,7 @@
       </c>
       <c r="M240" t="inlineStr"/>
       <c r="N240" t="inlineStr"/>
+      <c r="O240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -9975,6 +10219,7 @@
       </c>
       <c r="M241" t="inlineStr"/>
       <c r="N241" t="inlineStr"/>
+      <c r="O241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -10015,6 +10260,7 @@
       </c>
       <c r="M242" t="inlineStr"/>
       <c r="N242" t="inlineStr"/>
+      <c r="O242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -10055,6 +10301,7 @@
       </c>
       <c r="M243" t="inlineStr"/>
       <c r="N243" t="inlineStr"/>
+      <c r="O243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -10095,6 +10342,7 @@
       </c>
       <c r="M244" t="inlineStr"/>
       <c r="N244" t="inlineStr"/>
+      <c r="O244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -10135,6 +10383,7 @@
       </c>
       <c r="M245" t="inlineStr"/>
       <c r="N245" t="inlineStr"/>
+      <c r="O245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -10175,6 +10424,7 @@
       </c>
       <c r="M246" t="inlineStr"/>
       <c r="N246" t="inlineStr"/>
+      <c r="O246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -10215,6 +10465,7 @@
       </c>
       <c r="M247" t="inlineStr"/>
       <c r="N247" t="inlineStr"/>
+      <c r="O247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -10255,6 +10506,7 @@
       </c>
       <c r="M248" t="inlineStr"/>
       <c r="N248" t="inlineStr"/>
+      <c r="O248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -10295,6 +10547,7 @@
       </c>
       <c r="M249" t="inlineStr"/>
       <c r="N249" t="inlineStr"/>
+      <c r="O249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -10335,6 +10588,7 @@
       </c>
       <c r="M250" t="inlineStr"/>
       <c r="N250" t="inlineStr"/>
+      <c r="O250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -10375,6 +10629,7 @@
       </c>
       <c r="M251" t="inlineStr"/>
       <c r="N251" t="inlineStr"/>
+      <c r="O251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -10415,6 +10670,7 @@
       </c>
       <c r="M252" t="inlineStr"/>
       <c r="N252" t="inlineStr"/>
+      <c r="O252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -10455,6 +10711,7 @@
       </c>
       <c r="M253" t="inlineStr"/>
       <c r="N253" t="inlineStr"/>
+      <c r="O253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -10495,6 +10752,7 @@
       </c>
       <c r="M254" t="inlineStr"/>
       <c r="N254" t="inlineStr"/>
+      <c r="O254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -10535,6 +10793,7 @@
       </c>
       <c r="M255" t="inlineStr"/>
       <c r="N255" t="inlineStr"/>
+      <c r="O255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -10575,6 +10834,7 @@
       </c>
       <c r="M256" t="inlineStr"/>
       <c r="N256" t="inlineStr"/>
+      <c r="O256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -10611,6 +10871,7 @@
       <c r="L257" t="inlineStr"/>
       <c r="M257" t="inlineStr"/>
       <c r="N257" t="inlineStr"/>
+      <c r="O257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -10651,6 +10912,7 @@
       </c>
       <c r="M258" t="inlineStr"/>
       <c r="N258" t="inlineStr"/>
+      <c r="O258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -10691,6 +10953,7 @@
       </c>
       <c r="M259" t="inlineStr"/>
       <c r="N259" t="inlineStr"/>
+      <c r="O259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -10731,6 +10994,7 @@
       </c>
       <c r="M260" t="inlineStr"/>
       <c r="N260" t="inlineStr"/>
+      <c r="O260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -10771,6 +11035,7 @@
       </c>
       <c r="M261" t="inlineStr"/>
       <c r="N261" t="inlineStr"/>
+      <c r="O261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -10811,6 +11076,7 @@
       </c>
       <c r="M262" t="inlineStr"/>
       <c r="N262" t="inlineStr"/>
+      <c r="O262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -10847,6 +11113,7 @@
       <c r="L263" t="inlineStr"/>
       <c r="M263" t="inlineStr"/>
       <c r="N263" t="inlineStr"/>
+      <c r="O263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -10887,6 +11154,7 @@
       </c>
       <c r="M264" t="inlineStr"/>
       <c r="N264" t="inlineStr"/>
+      <c r="O264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -10927,6 +11195,7 @@
       </c>
       <c r="M265" t="inlineStr"/>
       <c r="N265" t="inlineStr"/>
+      <c r="O265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -10967,6 +11236,7 @@
       </c>
       <c r="M266" t="inlineStr"/>
       <c r="N266" t="inlineStr"/>
+      <c r="O266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -11007,6 +11277,7 @@
       </c>
       <c r="M267" t="inlineStr"/>
       <c r="N267" t="inlineStr"/>
+      <c r="O267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -11047,6 +11318,7 @@
       </c>
       <c r="M268" t="inlineStr"/>
       <c r="N268" t="inlineStr"/>
+      <c r="O268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -11087,6 +11359,7 @@
       </c>
       <c r="M269" t="inlineStr"/>
       <c r="N269" t="inlineStr"/>
+      <c r="O269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -11127,6 +11400,7 @@
       </c>
       <c r="M270" t="inlineStr"/>
       <c r="N270" t="inlineStr"/>
+      <c r="O270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -11167,6 +11441,7 @@
       </c>
       <c r="M271" t="inlineStr"/>
       <c r="N271" t="inlineStr"/>
+      <c r="O271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -11203,6 +11478,7 @@
       <c r="L272" t="inlineStr"/>
       <c r="M272" t="inlineStr"/>
       <c r="N272" t="inlineStr"/>
+      <c r="O272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -11243,6 +11519,7 @@
       </c>
       <c r="M273" t="inlineStr"/>
       <c r="N273" t="inlineStr"/>
+      <c r="O273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -11279,6 +11556,7 @@
       <c r="L274" t="inlineStr"/>
       <c r="M274" t="inlineStr"/>
       <c r="N274" t="inlineStr"/>
+      <c r="O274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -11319,6 +11597,7 @@
       </c>
       <c r="M275" t="inlineStr"/>
       <c r="N275" t="inlineStr"/>
+      <c r="O275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -11359,6 +11638,7 @@
       </c>
       <c r="M276" t="inlineStr"/>
       <c r="N276" t="inlineStr"/>
+      <c r="O276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -11399,6 +11679,7 @@
       </c>
       <c r="M277" t="inlineStr"/>
       <c r="N277" t="inlineStr"/>
+      <c r="O277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -11439,6 +11720,7 @@
       </c>
       <c r="M278" t="inlineStr"/>
       <c r="N278" t="inlineStr"/>
+      <c r="O278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -11479,6 +11761,7 @@
       </c>
       <c r="M279" t="inlineStr"/>
       <c r="N279" t="inlineStr"/>
+      <c r="O279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -11515,6 +11798,7 @@
       <c r="L280" t="inlineStr"/>
       <c r="M280" t="inlineStr"/>
       <c r="N280" t="inlineStr"/>
+      <c r="O280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -11555,6 +11839,7 @@
       </c>
       <c r="M281" t="inlineStr"/>
       <c r="N281" t="inlineStr"/>
+      <c r="O281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -11595,6 +11880,7 @@
       </c>
       <c r="M282" t="inlineStr"/>
       <c r="N282" t="inlineStr"/>
+      <c r="O282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -11635,6 +11921,7 @@
       </c>
       <c r="M283" t="inlineStr"/>
       <c r="N283" t="inlineStr"/>
+      <c r="O283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -11675,6 +11962,7 @@
       </c>
       <c r="M284" t="inlineStr"/>
       <c r="N284" t="inlineStr"/>
+      <c r="O284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -11707,6 +11995,7 @@
       <c r="L285" t="inlineStr"/>
       <c r="M285" t="inlineStr"/>
       <c r="N285" t="inlineStr"/>
+      <c r="O285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -11747,6 +12036,7 @@
       </c>
       <c r="M286" t="inlineStr"/>
       <c r="N286" t="inlineStr"/>
+      <c r="O286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -11783,6 +12073,7 @@
       <c r="L287" t="inlineStr"/>
       <c r="M287" t="inlineStr"/>
       <c r="N287" t="inlineStr"/>
+      <c r="O287" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -11823,6 +12114,7 @@
       </c>
       <c r="M288" t="inlineStr"/>
       <c r="N288" t="inlineStr"/>
+      <c r="O288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -11863,6 +12155,7 @@
       </c>
       <c r="M289" t="inlineStr"/>
       <c r="N289" t="inlineStr"/>
+      <c r="O289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -11903,6 +12196,7 @@
       </c>
       <c r="M290" t="inlineStr"/>
       <c r="N290" t="inlineStr"/>
+      <c r="O290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -11943,6 +12237,7 @@
       </c>
       <c r="M291" t="inlineStr"/>
       <c r="N291" t="inlineStr"/>
+      <c r="O291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -11979,6 +12274,7 @@
       <c r="L292" t="inlineStr"/>
       <c r="M292" t="inlineStr"/>
       <c r="N292" t="inlineStr"/>
+      <c r="O292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -12019,6 +12315,7 @@
       </c>
       <c r="M293" t="inlineStr"/>
       <c r="N293" t="inlineStr"/>
+      <c r="O293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -12059,6 +12356,7 @@
       </c>
       <c r="M294" t="inlineStr"/>
       <c r="N294" t="inlineStr"/>
+      <c r="O294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -12099,6 +12397,7 @@
       </c>
       <c r="M295" t="inlineStr"/>
       <c r="N295" t="inlineStr"/>
+      <c r="O295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -12139,6 +12438,7 @@
       </c>
       <c r="M296" t="inlineStr"/>
       <c r="N296" t="inlineStr"/>
+      <c r="O296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -12175,6 +12475,7 @@
       <c r="L297" t="inlineStr"/>
       <c r="M297" t="inlineStr"/>
       <c r="N297" t="inlineStr"/>
+      <c r="O297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -12211,6 +12512,7 @@
       <c r="L298" t="inlineStr"/>
       <c r="M298" t="inlineStr"/>
       <c r="N298" t="inlineStr"/>
+      <c r="O298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -12247,6 +12549,7 @@
       <c r="L299" t="inlineStr"/>
       <c r="M299" t="inlineStr"/>
       <c r="N299" t="inlineStr"/>
+      <c r="O299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -12287,6 +12590,7 @@
       </c>
       <c r="M300" t="inlineStr"/>
       <c r="N300" t="inlineStr"/>
+      <c r="O300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -12327,6 +12631,7 @@
       </c>
       <c r="M301" t="inlineStr"/>
       <c r="N301" t="inlineStr"/>
+      <c r="O301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -12367,6 +12672,7 @@
       </c>
       <c r="M302" t="inlineStr"/>
       <c r="N302" t="inlineStr"/>
+      <c r="O302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -12403,6 +12709,7 @@
       <c r="L303" t="inlineStr"/>
       <c r="M303" t="inlineStr"/>
       <c r="N303" t="inlineStr"/>
+      <c r="O303" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -12443,6 +12750,7 @@
       </c>
       <c r="M304" t="inlineStr"/>
       <c r="N304" t="inlineStr"/>
+      <c r="O304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -12483,6 +12791,7 @@
       </c>
       <c r="M305" t="inlineStr"/>
       <c r="N305" t="inlineStr"/>
+      <c r="O305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -12519,6 +12828,7 @@
       <c r="L306" t="inlineStr"/>
       <c r="M306" t="inlineStr"/>
       <c r="N306" t="inlineStr"/>
+      <c r="O306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -12559,6 +12869,7 @@
       </c>
       <c r="M307" t="inlineStr"/>
       <c r="N307" t="inlineStr"/>
+      <c r="O307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -12595,6 +12906,7 @@
       <c r="L308" t="inlineStr"/>
       <c r="M308" t="inlineStr"/>
       <c r="N308" t="inlineStr"/>
+      <c r="O308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -12635,6 +12947,7 @@
       </c>
       <c r="M309" t="inlineStr"/>
       <c r="N309" t="inlineStr"/>
+      <c r="O309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -12671,6 +12984,7 @@
       <c r="L310" t="inlineStr"/>
       <c r="M310" t="inlineStr"/>
       <c r="N310" t="inlineStr"/>
+      <c r="O310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -12711,6 +13025,7 @@
       </c>
       <c r="M311" t="inlineStr"/>
       <c r="N311" t="inlineStr"/>
+      <c r="O311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -12751,6 +13066,7 @@
       </c>
       <c r="M312" t="inlineStr"/>
       <c r="N312" t="inlineStr"/>
+      <c r="O312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -12791,6 +13107,7 @@
       </c>
       <c r="M313" t="inlineStr"/>
       <c r="N313" t="inlineStr"/>
+      <c r="O313" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -12831,6 +13148,7 @@
       </c>
       <c r="M314" t="inlineStr"/>
       <c r="N314" t="inlineStr"/>
+      <c r="O314" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -12871,6 +13189,7 @@
       </c>
       <c r="M315" t="inlineStr"/>
       <c r="N315" t="inlineStr"/>
+      <c r="O315" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -12911,6 +13230,7 @@
       </c>
       <c r="M316" t="inlineStr"/>
       <c r="N316" t="inlineStr"/>
+      <c r="O316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -12951,6 +13271,7 @@
       </c>
       <c r="M317" t="inlineStr"/>
       <c r="N317" t="inlineStr"/>
+      <c r="O317" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -12991,6 +13312,7 @@
       </c>
       <c r="M318" t="inlineStr"/>
       <c r="N318" t="inlineStr"/>
+      <c r="O318" t="inlineStr"/>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -13031,6 +13353,7 @@
       </c>
       <c r="M319" t="inlineStr"/>
       <c r="N319" t="inlineStr"/>
+      <c r="O319" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -13067,6 +13390,7 @@
       <c r="L320" t="inlineStr"/>
       <c r="M320" t="inlineStr"/>
       <c r="N320" t="inlineStr"/>
+      <c r="O320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -13107,6 +13431,7 @@
       </c>
       <c r="M321" t="inlineStr"/>
       <c r="N321" t="inlineStr"/>
+      <c r="O321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -13147,6 +13472,7 @@
       </c>
       <c r="M322" t="inlineStr"/>
       <c r="N322" t="inlineStr"/>
+      <c r="O322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -13183,6 +13509,7 @@
       <c r="L323" t="inlineStr"/>
       <c r="M323" t="inlineStr"/>
       <c r="N323" t="inlineStr"/>
+      <c r="O323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -13223,6 +13550,7 @@
       </c>
       <c r="M324" t="inlineStr"/>
       <c r="N324" t="inlineStr"/>
+      <c r="O324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -13263,6 +13591,7 @@
       </c>
       <c r="M325" t="inlineStr"/>
       <c r="N325" t="inlineStr"/>
+      <c r="O325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -13303,6 +13632,7 @@
       </c>
       <c r="M326" t="inlineStr"/>
       <c r="N326" t="inlineStr"/>
+      <c r="O326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -13343,6 +13673,7 @@
       </c>
       <c r="M327" t="inlineStr"/>
       <c r="N327" t="inlineStr"/>
+      <c r="O327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -13383,6 +13714,7 @@
       </c>
       <c r="M328" t="inlineStr"/>
       <c r="N328" t="inlineStr"/>
+      <c r="O328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -13419,6 +13751,7 @@
       <c r="L329" t="inlineStr"/>
       <c r="M329" t="inlineStr"/>
       <c r="N329" t="inlineStr"/>
+      <c r="O329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -13459,6 +13792,7 @@
       </c>
       <c r="M330" t="inlineStr"/>
       <c r="N330" t="inlineStr"/>
+      <c r="O330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -13499,6 +13833,7 @@
       </c>
       <c r="M331" t="inlineStr"/>
       <c r="N331" t="inlineStr"/>
+      <c r="O331" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -13539,6 +13874,7 @@
       </c>
       <c r="M332" t="inlineStr"/>
       <c r="N332" t="inlineStr"/>
+      <c r="O332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -13579,6 +13915,7 @@
       </c>
       <c r="M333" t="inlineStr"/>
       <c r="N333" t="inlineStr"/>
+      <c r="O333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -13619,6 +13956,7 @@
       </c>
       <c r="M334" t="inlineStr"/>
       <c r="N334" t="inlineStr"/>
+      <c r="O334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -13659,6 +13997,7 @@
       </c>
       <c r="M335" t="inlineStr"/>
       <c r="N335" t="inlineStr"/>
+      <c r="O335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -13699,6 +14038,7 @@
       </c>
       <c r="M336" t="inlineStr"/>
       <c r="N336" t="inlineStr"/>
+      <c r="O336" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -13735,6 +14075,7 @@
       <c r="L337" t="inlineStr"/>
       <c r="M337" t="inlineStr"/>
       <c r="N337" t="inlineStr"/>
+      <c r="O337" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -13775,6 +14116,7 @@
       </c>
       <c r="M338" t="inlineStr"/>
       <c r="N338" t="inlineStr"/>
+      <c r="O338" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -13815,6 +14157,7 @@
       </c>
       <c r="M339" t="inlineStr"/>
       <c r="N339" t="inlineStr"/>
+      <c r="O339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -13851,6 +14194,7 @@
       <c r="L340" t="inlineStr"/>
       <c r="M340" t="inlineStr"/>
       <c r="N340" t="inlineStr"/>
+      <c r="O340" t="inlineStr"/>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -13891,6 +14235,7 @@
       </c>
       <c r="M341" t="inlineStr"/>
       <c r="N341" t="inlineStr"/>
+      <c r="O341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -13931,6 +14276,7 @@
       </c>
       <c r="M342" t="inlineStr"/>
       <c r="N342" t="inlineStr"/>
+      <c r="O342" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -13971,6 +14317,7 @@
       </c>
       <c r="M343" t="inlineStr"/>
       <c r="N343" t="inlineStr"/>
+      <c r="O343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -14011,6 +14358,7 @@
       </c>
       <c r="M344" t="inlineStr"/>
       <c r="N344" t="inlineStr"/>
+      <c r="O344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -14047,6 +14395,7 @@
       <c r="L345" t="inlineStr"/>
       <c r="M345" t="inlineStr"/>
       <c r="N345" t="inlineStr"/>
+      <c r="O345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -14087,6 +14436,7 @@
       </c>
       <c r="M346" t="inlineStr"/>
       <c r="N346" t="inlineStr"/>
+      <c r="O346" t="inlineStr"/>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -14127,6 +14477,7 @@
       </c>
       <c r="M347" t="inlineStr"/>
       <c r="N347" t="inlineStr"/>
+      <c r="O347" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -14167,6 +14518,7 @@
       </c>
       <c r="M348" t="inlineStr"/>
       <c r="N348" t="inlineStr"/>
+      <c r="O348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -14203,6 +14555,7 @@
       <c r="L349" t="inlineStr"/>
       <c r="M349" t="inlineStr"/>
       <c r="N349" t="inlineStr"/>
+      <c r="O349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -14243,6 +14596,7 @@
       </c>
       <c r="M350" t="inlineStr"/>
       <c r="N350" t="inlineStr"/>
+      <c r="O350" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -14283,6 +14637,7 @@
       </c>
       <c r="M351" t="inlineStr"/>
       <c r="N351" t="inlineStr"/>
+      <c r="O351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -14323,6 +14678,7 @@
       </c>
       <c r="M352" t="inlineStr"/>
       <c r="N352" t="inlineStr"/>
+      <c r="O352" t="inlineStr"/>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -14363,6 +14719,7 @@
       </c>
       <c r="M353" t="inlineStr"/>
       <c r="N353" t="inlineStr"/>
+      <c r="O353" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -14403,6 +14760,7 @@
       </c>
       <c r="M354" t="inlineStr"/>
       <c r="N354" t="inlineStr"/>
+      <c r="O354" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -14443,6 +14801,7 @@
       </c>
       <c r="M355" t="inlineStr"/>
       <c r="N355" t="inlineStr"/>
+      <c r="O355" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -14483,6 +14842,7 @@
       </c>
       <c r="M356" t="inlineStr"/>
       <c r="N356" t="inlineStr"/>
+      <c r="O356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -14523,6 +14883,7 @@
       </c>
       <c r="M357" t="inlineStr"/>
       <c r="N357" t="inlineStr"/>
+      <c r="O357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -14559,6 +14920,7 @@
       <c r="L358" t="inlineStr"/>
       <c r="M358" t="inlineStr"/>
       <c r="N358" t="inlineStr"/>
+      <c r="O358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -14599,6 +14961,7 @@
       </c>
       <c r="M359" t="inlineStr"/>
       <c r="N359" t="inlineStr"/>
+      <c r="O359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -14639,6 +15002,7 @@
       </c>
       <c r="M360" t="inlineStr"/>
       <c r="N360" t="inlineStr"/>
+      <c r="O360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -14679,6 +15043,7 @@
       </c>
       <c r="M361" t="inlineStr"/>
       <c r="N361" t="inlineStr"/>
+      <c r="O361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -14719,6 +15084,7 @@
       </c>
       <c r="M362" t="inlineStr"/>
       <c r="N362" t="inlineStr"/>
+      <c r="O362" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -14759,6 +15125,7 @@
       </c>
       <c r="M363" t="inlineStr"/>
       <c r="N363" t="inlineStr"/>
+      <c r="O363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -14795,6 +15162,7 @@
       <c r="L364" t="inlineStr"/>
       <c r="M364" t="inlineStr"/>
       <c r="N364" t="inlineStr"/>
+      <c r="O364" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -14831,6 +15199,7 @@
       <c r="L365" t="inlineStr"/>
       <c r="M365" t="inlineStr"/>
       <c r="N365" t="inlineStr"/>
+      <c r="O365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -14871,6 +15240,7 @@
       </c>
       <c r="M366" t="inlineStr"/>
       <c r="N366" t="inlineStr"/>
+      <c r="O366" t="inlineStr"/>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -14911,6 +15281,7 @@
       </c>
       <c r="M367" t="inlineStr"/>
       <c r="N367" t="inlineStr"/>
+      <c r="O367" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -14947,6 +15318,7 @@
       <c r="L368" t="inlineStr"/>
       <c r="M368" t="inlineStr"/>
       <c r="N368" t="inlineStr"/>
+      <c r="O368" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -14987,6 +15359,7 @@
       </c>
       <c r="M369" t="inlineStr"/>
       <c r="N369" t="inlineStr"/>
+      <c r="O369" t="inlineStr"/>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -15027,6 +15400,7 @@
       </c>
       <c r="M370" t="inlineStr"/>
       <c r="N370" t="inlineStr"/>
+      <c r="O370" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -15067,6 +15441,7 @@
       </c>
       <c r="M371" t="inlineStr"/>
       <c r="N371" t="inlineStr"/>
+      <c r="O371" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -15107,6 +15482,7 @@
       </c>
       <c r="M372" t="inlineStr"/>
       <c r="N372" t="inlineStr"/>
+      <c r="O372" t="inlineStr"/>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -15143,6 +15519,7 @@
       <c r="L373" t="inlineStr"/>
       <c r="M373" t="inlineStr"/>
       <c r="N373" t="inlineStr"/>
+      <c r="O373" t="inlineStr"/>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
@@ -15183,6 +15560,7 @@
       </c>
       <c r="M374" t="inlineStr"/>
       <c r="N374" t="inlineStr"/>
+      <c r="O374" t="inlineStr"/>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -15223,6 +15601,7 @@
       </c>
       <c r="M375" t="inlineStr"/>
       <c r="N375" t="inlineStr"/>
+      <c r="O375" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -15263,6 +15642,7 @@
       </c>
       <c r="M376" t="inlineStr"/>
       <c r="N376" t="inlineStr"/>
+      <c r="O376" t="inlineStr"/>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -15303,6 +15683,7 @@
       </c>
       <c r="M377" t="inlineStr"/>
       <c r="N377" t="inlineStr"/>
+      <c r="O377" t="inlineStr"/>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -15343,6 +15724,7 @@
       </c>
       <c r="M378" t="inlineStr"/>
       <c r="N378" t="inlineStr"/>
+      <c r="O378" t="inlineStr"/>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -15379,6 +15761,7 @@
       <c r="L379" t="inlineStr"/>
       <c r="M379" t="inlineStr"/>
       <c r="N379" t="inlineStr"/>
+      <c r="O379" t="inlineStr"/>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -15415,6 +15798,7 @@
       <c r="L380" t="inlineStr"/>
       <c r="M380" t="inlineStr"/>
       <c r="N380" t="inlineStr"/>
+      <c r="O380" t="inlineStr"/>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
@@ -15451,6 +15835,7 @@
       <c r="L381" t="inlineStr"/>
       <c r="M381" t="inlineStr"/>
       <c r="N381" t="inlineStr"/>
+      <c r="O381" t="inlineStr"/>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -15487,6 +15872,7 @@
       <c r="L382" t="inlineStr"/>
       <c r="M382" t="inlineStr"/>
       <c r="N382" t="inlineStr"/>
+      <c r="O382" t="inlineStr"/>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -15527,6 +15913,7 @@
       </c>
       <c r="M383" t="inlineStr"/>
       <c r="N383" t="inlineStr"/>
+      <c r="O383" t="inlineStr"/>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
@@ -15567,6 +15954,7 @@
       </c>
       <c r="M384" t="inlineStr"/>
       <c r="N384" t="inlineStr"/>
+      <c r="O384" t="inlineStr"/>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
@@ -15607,6 +15995,7 @@
       </c>
       <c r="M385" t="inlineStr"/>
       <c r="N385" t="inlineStr"/>
+      <c r="O385" t="inlineStr"/>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
@@ -15647,6 +16036,7 @@
       </c>
       <c r="M386" t="inlineStr"/>
       <c r="N386" t="inlineStr"/>
+      <c r="O386" t="inlineStr"/>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
@@ -15687,6 +16077,7 @@
       </c>
       <c r="M387" t="inlineStr"/>
       <c r="N387" t="inlineStr"/>
+      <c r="O387" t="inlineStr"/>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -15727,6 +16118,7 @@
       </c>
       <c r="M388" t="inlineStr"/>
       <c r="N388" t="inlineStr"/>
+      <c r="O388" t="inlineStr"/>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -15767,6 +16159,7 @@
       </c>
       <c r="M389" t="inlineStr"/>
       <c r="N389" t="inlineStr"/>
+      <c r="O389" t="inlineStr"/>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
@@ -15807,6 +16200,7 @@
       </c>
       <c r="M390" t="inlineStr"/>
       <c r="N390" t="inlineStr"/>
+      <c r="O390" t="inlineStr"/>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
@@ -15839,6 +16233,7 @@
       <c r="L391" t="inlineStr"/>
       <c r="M391" t="inlineStr"/>
       <c r="N391" t="inlineStr"/>
+      <c r="O391" t="inlineStr"/>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
@@ -15879,6 +16274,7 @@
       </c>
       <c r="M392" t="inlineStr"/>
       <c r="N392" t="inlineStr"/>
+      <c r="O392" t="inlineStr"/>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
@@ -15919,6 +16315,7 @@
       </c>
       <c r="M393" t="inlineStr"/>
       <c r="N393" t="inlineStr"/>
+      <c r="O393" t="inlineStr"/>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -15959,6 +16356,7 @@
       </c>
       <c r="M394" t="inlineStr"/>
       <c r="N394" t="inlineStr"/>
+      <c r="O394" t="inlineStr"/>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
@@ -15999,6 +16397,7 @@
       </c>
       <c r="M395" t="inlineStr"/>
       <c r="N395" t="inlineStr"/>
+      <c r="O395" t="inlineStr"/>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
@@ -16039,6 +16438,7 @@
       </c>
       <c r="M396" t="inlineStr"/>
       <c r="N396" t="inlineStr"/>
+      <c r="O396" t="inlineStr"/>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -16079,6 +16479,7 @@
       </c>
       <c r="M397" t="inlineStr"/>
       <c r="N397" t="inlineStr"/>
+      <c r="O397" t="inlineStr"/>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -16115,6 +16516,7 @@
       <c r="L398" t="inlineStr"/>
       <c r="M398" t="inlineStr"/>
       <c r="N398" t="inlineStr"/>
+      <c r="O398" t="inlineStr"/>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
@@ -16155,6 +16557,7 @@
       </c>
       <c r="M399" t="inlineStr"/>
       <c r="N399" t="inlineStr"/>
+      <c r="O399" t="inlineStr"/>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -16195,6 +16598,7 @@
       </c>
       <c r="M400" t="inlineStr"/>
       <c r="N400" t="inlineStr"/>
+      <c r="O400" t="inlineStr"/>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
@@ -16235,6 +16639,7 @@
       </c>
       <c r="M401" t="inlineStr"/>
       <c r="N401" t="inlineStr"/>
+      <c r="O401" t="inlineStr"/>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
@@ -16275,6 +16680,7 @@
       </c>
       <c r="M402" t="inlineStr"/>
       <c r="N402" t="inlineStr"/>
+      <c r="O402" t="inlineStr"/>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
@@ -16315,6 +16721,7 @@
       </c>
       <c r="M403" t="inlineStr"/>
       <c r="N403" t="inlineStr"/>
+      <c r="O403" t="inlineStr"/>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
@@ -16351,6 +16758,7 @@
       <c r="L404" t="inlineStr"/>
       <c r="M404" t="inlineStr"/>
       <c r="N404" t="inlineStr"/>
+      <c r="O404" t="inlineStr"/>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
@@ -16391,6 +16799,7 @@
       </c>
       <c r="M405" t="inlineStr"/>
       <c r="N405" t="inlineStr"/>
+      <c r="O405" t="inlineStr"/>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
@@ -16431,6 +16840,7 @@
       </c>
       <c r="M406" t="inlineStr"/>
       <c r="N406" t="inlineStr"/>
+      <c r="O406" t="inlineStr"/>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
@@ -16467,6 +16877,7 @@
       <c r="L407" t="inlineStr"/>
       <c r="M407" t="inlineStr"/>
       <c r="N407" t="inlineStr"/>
+      <c r="O407" t="inlineStr"/>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
@@ -16523,10 +16934,15 @@
       </c>
       <c r="M408" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Vehículos y Equipo Terrestre</t>
         </is>
       </c>
       <c r="N408" t="inlineStr">
+        <is>
+          <t>la Procuraduría General de Justicia del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O408" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0407-2026.pdf</t>
         </is>
@@ -16567,6 +16983,7 @@
       <c r="L409" t="inlineStr"/>
       <c r="M409" t="inlineStr"/>
       <c r="N409" t="inlineStr"/>
+      <c r="O409" t="inlineStr"/>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
@@ -16607,6 +17024,7 @@
       </c>
       <c r="M410" t="inlineStr"/>
       <c r="N410" t="inlineStr"/>
+      <c r="O410" t="inlineStr"/>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
@@ -16647,6 +17065,7 @@
       </c>
       <c r="M411" t="inlineStr"/>
       <c r="N411" t="inlineStr"/>
+      <c r="O411" t="inlineStr"/>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
@@ -16683,6 +17102,7 @@
       <c r="L412" t="inlineStr"/>
       <c r="M412" t="inlineStr"/>
       <c r="N412" t="inlineStr"/>
+      <c r="O412" t="inlineStr"/>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
@@ -16723,6 +17143,7 @@
       </c>
       <c r="M413" t="inlineStr"/>
       <c r="N413" t="inlineStr"/>
+      <c r="O413" t="inlineStr"/>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
@@ -16763,6 +17184,7 @@
       </c>
       <c r="M414" t="inlineStr"/>
       <c r="N414" t="inlineStr"/>
+      <c r="O414" t="inlineStr"/>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
@@ -16803,6 +17225,7 @@
       </c>
       <c r="M415" t="inlineStr"/>
       <c r="N415" t="inlineStr"/>
+      <c r="O415" t="inlineStr"/>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
@@ -16839,6 +17262,7 @@
       <c r="L416" t="inlineStr"/>
       <c r="M416" t="inlineStr"/>
       <c r="N416" t="inlineStr"/>
+      <c r="O416" t="inlineStr"/>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
@@ -16875,6 +17299,7 @@
       <c r="L417" t="inlineStr"/>
       <c r="M417" t="inlineStr"/>
       <c r="N417" t="inlineStr"/>
+      <c r="O417" t="inlineStr"/>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
@@ -16911,6 +17336,7 @@
       <c r="L418" t="inlineStr"/>
       <c r="M418" t="inlineStr"/>
       <c r="N418" t="inlineStr"/>
+      <c r="O418" t="inlineStr"/>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
@@ -16947,6 +17373,7 @@
       <c r="L419" t="inlineStr"/>
       <c r="M419" t="inlineStr"/>
       <c r="N419" t="inlineStr"/>
+      <c r="O419" t="inlineStr"/>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
@@ -16987,6 +17414,7 @@
       </c>
       <c r="M420" t="inlineStr"/>
       <c r="N420" t="inlineStr"/>
+      <c r="O420" t="inlineStr"/>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
@@ -17019,6 +17447,7 @@
       <c r="L421" t="inlineStr"/>
       <c r="M421" t="inlineStr"/>
       <c r="N421" t="inlineStr"/>
+      <c r="O421" t="inlineStr"/>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
@@ -17051,6 +17480,7 @@
       <c r="L422" t="inlineStr"/>
       <c r="M422" t="inlineStr"/>
       <c r="N422" t="inlineStr"/>
+      <c r="O422" t="inlineStr"/>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
@@ -17083,6 +17513,7 @@
       <c r="L423" t="inlineStr"/>
       <c r="M423" t="inlineStr"/>
       <c r="N423" t="inlineStr"/>
+      <c r="O423" t="inlineStr"/>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
@@ -17131,10 +17562,15 @@
       <c r="L424" t="inlineStr"/>
       <c r="M424" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Activos Intangibles (Sistema Integral de Enseñanza, aprendizaje y certificación del idioma inglés)</t>
         </is>
       </c>
       <c r="N424" t="inlineStr">
+        <is>
+          <t>el Instituto Tecnológico Superior de Huichapan</t>
+        </is>
+      </c>
+      <c r="O424" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0423-2026.pdf</t>
         </is>
@@ -17187,10 +17623,15 @@
       <c r="L425" t="inlineStr"/>
       <c r="M425" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Vestuario y Uniformes</t>
         </is>
       </c>
       <c r="N425" t="inlineStr">
+        <is>
+          <t>la Subsecretaría de Operación Policial de la Secretaría de Seguridad Pública del Poder Ejecutivo del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O425" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0424-2026.pdf</t>
         </is>
@@ -17243,10 +17684,15 @@
       <c r="L426" t="inlineStr"/>
       <c r="M426" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Otros Materiales y Artículos de Construcción y Reparación</t>
         </is>
       </c>
       <c r="N426" t="inlineStr">
+        <is>
+          <t>la Dirección General de Conservación de Carreteras Estatales de la Secretaría de Infraestructura Pública y Desarrollo Urbano Sostenible del Poder Ejecutivo del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O426" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0425-2026.pdf</t>
         </is>
@@ -17299,10 +17745,15 @@
       <c r="L427" t="inlineStr"/>
       <c r="M427" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Material de Oficina, Materiales y Útiles Consumibles para el Procesamiento en Equipos y Bienes Informáticos, Material de Limpieza</t>
         </is>
       </c>
       <c r="N427" t="inlineStr">
+        <is>
+          <t>la Dirección General de Conservación de Carreteras Estatales de la Secretaría de Infraestructura Pública y Desarrollo Urbano Sostenible del Poder Ejecutivo del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O427" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0426-2026.pdf</t>
         </is>
@@ -17355,10 +17806,15 @@
       <c r="L428" t="inlineStr"/>
       <c r="M428" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Combustibles y Lubricantes para Vehículos y Equipos Terrestres, Refacciones para Vehículos y Equipos de Transporte</t>
         </is>
       </c>
       <c r="N428" t="inlineStr">
+        <is>
+          <t>la Dirección General de Conservación de Carreteras Estatales de la Secretaría de Infraestructura Pública y Desarrollo Urbano Sostenible del Poder Ejecutivo del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O428" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0427-2026.pdf</t>
         </is>
@@ -17411,10 +17867,15 @@
       <c r="L429" t="inlineStr"/>
       <c r="M429" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Prendas de Seguridad y Protección Personal, Identificadores e Iconos de Señalización, Herramientas Menores</t>
         </is>
       </c>
       <c r="N429" t="inlineStr">
+        <is>
+          <t>la Dirección General de Conservación de Carreteras Estatales de la Secretaría de Infraestructura Pública y Desarrollo Urbano Sostenible del Poder Ejecutivo del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O429" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0428-2026.pdf</t>
         </is>
@@ -17467,10 +17928,15 @@
       <c r="L430" t="inlineStr"/>
       <c r="M430" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Arrendamiento de Maquinaria, Otros Equipos y Herramientas</t>
         </is>
       </c>
       <c r="N430" t="inlineStr">
+        <is>
+          <t>la Dirección General de Conservación de Carreteras Estatales de la Secretaría de Infraestructura Pública y Desarrollo Urbano Sostenible del Poder Ejecutivo del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O430" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0429-2026.pdf</t>
         </is>
@@ -17523,10 +17989,15 @@
       <c r="L431" t="inlineStr"/>
       <c r="M431" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Prendas de Seguridad y Protección Personal</t>
         </is>
       </c>
       <c r="N431" t="inlineStr">
+        <is>
+          <t>la Dirección General de Conservación de Carreteras Estatales de la Secretaría de Infraestructura Pública y Desarrollo Urbano Sostenible del Poder Ejecutivo del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O431" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0430-2026.pdf</t>
         </is>
@@ -17571,10 +18042,15 @@
       <c r="L432" t="inlineStr"/>
       <c r="M432" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Uniformes Escolares</t>
         </is>
       </c>
       <c r="N432" t="inlineStr">
+        <is>
+          <t>el Colegio de Educación Profesional Técnica del Estado de Hidalgo, el Colegio de Bachilleres del Estado de Hidalgo, el Bachillerato del Estado de Hidalgo y el Colegio de Estudios Científicos y Tecnológicos del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O432" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0431-2026.pdf</t>
         </is>
@@ -17627,10 +18103,15 @@
       <c r="L433" t="inlineStr"/>
       <c r="M433" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Asignación de Combustible a través de Monederos Electrónicos</t>
         </is>
       </c>
       <c r="N433" t="inlineStr">
+        <is>
+          <t>la Dirección General de Conservación de Carreteras Estatales de la Secretaría de Infraestructura Pública y Desarrollo Urbano Sostenible del Poder Ejecutivo del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O433" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0432-2026.pdf</t>
         </is>
@@ -17683,10 +18164,15 @@
       <c r="L434" t="inlineStr"/>
       <c r="M434" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Mantenimiento de Maquinaria y Equipo</t>
         </is>
       </c>
       <c r="N434" t="inlineStr">
+        <is>
+          <t>la Dirección General de Conservación de Carreteras Estatales de la Secretaría de Infraestructura Pública y Desarrollo Urbano Sostenible del Poder Ejecutivo del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O434" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0433-2026.pdf</t>
         </is>
@@ -17739,10 +18225,15 @@
       <c r="L435" t="inlineStr"/>
       <c r="M435" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Material Eléctrico, Artículos Metálicos para la Construcción</t>
         </is>
       </c>
       <c r="N435" t="inlineStr">
+        <is>
+          <t>la Procuraduría General de Justicia del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O435" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0434-2026.pdf</t>
         </is>
@@ -17795,10 +18286,15 @@
       <c r="L436" t="inlineStr"/>
       <c r="M436" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Artículos Metálicos para la Construcción, Otros Materiales y Artículos de Construcción y Reparación, Identificadores e Iconos De Señalización</t>
         </is>
       </c>
       <c r="N436" t="inlineStr">
+        <is>
+          <t>la Dirección General de Conservación de Carreteras Estatales de la Secretaría de Infraestructura Pública y Desarrollo Urbano Sostenible del Poder Ejecutivo del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O436" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0435-2026.pdf</t>
         </is>
@@ -17851,10 +18347,15 @@
       <c r="L437" t="inlineStr"/>
       <c r="M437" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Materiales y Útiles Consumibles para el Procesamiento en Equipos y Bienes Informáticos, Materiales para el Mantenimiento de Señalizaciones</t>
         </is>
       </c>
       <c r="N437" t="inlineStr">
+        <is>
+          <t>la Dirección General de Conservación de Carreteras Estatales de la Secretaría de Infraestructura Pública y Desarrollo Urbano Sostenible del Poder Ejecutivo del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O437" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0436-2026.pdf</t>
         </is>
@@ -17907,10 +18408,15 @@
       <c r="L438" t="inlineStr"/>
       <c r="M438" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Blancos y Otros Productos Textiles, Excepto Prendas de Vestir</t>
         </is>
       </c>
       <c r="N438" t="inlineStr">
+        <is>
+          <t>los Centros de Rehabilitación Integral Hidalgo del Sistema para el Desarrollo Integral de la Familia del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O438" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0437-2026.pdf</t>
         </is>
@@ -17959,10 +18465,15 @@
       <c r="L439" t="inlineStr"/>
       <c r="M439" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Servicios Integrales</t>
         </is>
       </c>
       <c r="N439" t="inlineStr">
+        <is>
+          <t>la Dirección General de Formación y Competitividad Turística de la Secretaría de Turismo del Poder Ejecutivo del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O439" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0438-2026.pdf</t>
         </is>
@@ -18011,10 +18522,15 @@
       <c r="L440" t="inlineStr"/>
       <c r="M440" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Servicios de Acceso de Internet, Redes y Procesamiento de Información</t>
         </is>
       </c>
       <c r="N440" t="inlineStr">
+        <is>
+          <t>la Dirección General de Prevención y Reinserción Social de la Secretaría de Seguridad Pública del Poder Ejecutivo del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O440" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0439-2026.pdf</t>
         </is>
@@ -18063,10 +18579,15 @@
       <c r="L441" t="inlineStr"/>
       <c r="M441" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Mantenimiento de Maquinaria y Equipo</t>
         </is>
       </c>
       <c r="N441" t="inlineStr">
+        <is>
+          <t>la Subsecretaria del Centro de Control, Comando, Comunicaciones, Cómputo, Coordinación, e Inteligencia de la Secretaría de Seguridad Pública del Poder Ejecutivo del Gobierno del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O441" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0440-2026.pdf</t>
         </is>
@@ -18115,10 +18636,15 @@
       <c r="L442" t="inlineStr"/>
       <c r="M442" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Materiales y Útiles Consumibles para el Procesamiento en Equipos y Bienes Informáticos</t>
         </is>
       </c>
       <c r="N442" t="inlineStr">
+        <is>
+          <t>la Subsecretaría de Inclusión y Desarrollo y la Subsecretaría de Participación Social y Fomento Artesanal de la Secretaría de Bienestar e Inclusión Social del Poder Ejecutivo del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O442" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0441-2026.pdf</t>
         </is>
@@ -18167,10 +18693,15 @@
       <c r="L443" t="inlineStr"/>
       <c r="M443" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Mantenimiento de Maquinaria y Equipo (Segundo Procedimiento)</t>
         </is>
       </c>
       <c r="N443" t="inlineStr">
+        <is>
+          <t>la Dirección General de Cuencas y Planeación Hídrica, de la Secretaría de Medio Ambiente y Recursos Naturales del Poder Ejecutivo del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O443" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0442-2026.pdf</t>
         </is>
@@ -18219,10 +18750,15 @@
       <c r="L444" t="inlineStr"/>
       <c r="M444" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Sustancias Químicas</t>
         </is>
       </c>
       <c r="N444" t="inlineStr">
+        <is>
+          <t>la Dirección General de Gestión de Calidad del Aire, de la Secretaría de Medio Ambiente y Recursos Naturales del Poder Ejecutivo del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O444" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0443-2026.pdf</t>
         </is>
@@ -18271,10 +18807,15 @@
       <c r="L445" t="inlineStr"/>
       <c r="M445" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Servicio de Fumigación</t>
         </is>
       </c>
       <c r="N445" t="inlineStr">
+        <is>
+          <t>la Dirección General de Recursos Materiales de la Oficialía Mayor del Gobierno del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O445" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0444-2026.pdf</t>
         </is>
@@ -18323,10 +18864,15 @@
       <c r="L446" t="inlineStr"/>
       <c r="M446" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Materiales, Accesorios y Suministros de Laboratorio, Refacciones y Accesorios Menores de Equipo e Instrumental Médico y de Laboratorio</t>
         </is>
       </c>
       <c r="N446" t="inlineStr">
+        <is>
+          <t>la Dirección General de Gestión de Calidad del Aire, de la Secretaría de Medio Ambiente y Recursos Naturales del Poder Ejecutivo del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O446" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0445-2026.pdf</t>
         </is>
@@ -18375,10 +18921,15 @@
       <c r="L447" t="inlineStr"/>
       <c r="M447" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Servicio de Fumigación</t>
         </is>
       </c>
       <c r="N447" t="inlineStr">
+        <is>
+          <t>la Secretaría del Trabajo y Previsión Social, Secretaría de Contraloría, Secretaría de Educación Pública, Secretaría de Seguridad Pública, Secretaría de Turismo, Secretaría de Desarrollo Económico, Secretaría de Medio Ambiente y Recursos Naturales, Secretaría de Agricultura y Desarrollo Rural, Unida</t>
+        </is>
+      </c>
+      <c r="O447" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0446-2026.pdf</t>
         </is>
@@ -18427,10 +18978,15 @@
       <c r="L448" t="inlineStr"/>
       <c r="M448" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Servicios Integrales (Segundo Procedimiento)</t>
         </is>
       </c>
       <c r="N448" t="inlineStr">
+        <is>
+          <t>la Universidad Tecnológica de Tulancingo</t>
+        </is>
+      </c>
+      <c r="O448" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0447-2026.pdf</t>
         </is>
@@ -18479,10 +19035,15 @@
       <c r="L449" t="inlineStr"/>
       <c r="M449" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Otros Arrendamientos para el evento “Viviendo en Plenitud”</t>
         </is>
       </c>
       <c r="N449" t="inlineStr">
+        <is>
+          <t>la Dirección de Asistencia Social del Sistema para el Desarrollo Integral de la Familia del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O449" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0448-2026.pdf</t>
         </is>
@@ -18531,10 +19092,15 @@
       <c r="L450" t="inlineStr"/>
       <c r="M450" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Servicio de Alimentos y Servicio de Impresiones para el evento “Viviendo en Plenitud”</t>
         </is>
       </c>
       <c r="N450" t="inlineStr">
+        <is>
+          <t>la Dirección de Asistencia Social del Sistema para el Desarrollo Integral de la Familia del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O450" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0449-2026.pdf</t>
         </is>
@@ -18583,10 +19149,15 @@
       <c r="L451" t="inlineStr"/>
       <c r="M451" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Equipo Médico y de Laboratorio (Electromiógrafo)</t>
         </is>
       </c>
       <c r="N451" t="inlineStr">
+        <is>
+          <t>el Hospital del Niño DIF Hidalgo del Sistema para el Desarrollo Integral de la Familia del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O451" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0450-2026.pdf</t>
         </is>
@@ -18635,10 +19206,15 @@
       <c r="L452" t="inlineStr"/>
       <c r="M452" t="inlineStr">
         <is>
-          <t>objeto de esta licitación.</t>
+          <t>Instrumental Médico y de Laboratorio</t>
         </is>
       </c>
       <c r="N452" t="inlineStr">
+        <is>
+          <t>el Hospital del Niño DIF Hidalgo del Sistema para el Desarrollo Integral de la Familia del Estado de Hidalgo</t>
+        </is>
+      </c>
+      <c r="O452" t="inlineStr">
         <is>
           <t>pdfs/EA-913003989-N0451-2026.pdf</t>
         </is>

</xml_diff>